<commit_message>
Add cpu_threshold to settings Excel file
Added cpu_threshold to settings Excel file and its corresponding import routine.
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F0B0AD-3F43-43B1-BD25-3077F07FFB27}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9988FBC5-74D5-463C-9BC8-F8F1D27B313A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>path_exe</t>
   </si>
@@ -112,6 +112,12 @@
   </si>
   <si>
     <t>name_excelsheet_sim_variants</t>
+  </si>
+  <si>
+    <t>cpu_threshold</t>
+  </si>
+  <si>
+    <t>CPU-Auslastung, welche unterschritten werden muss um die nächste Simulation zu starten</t>
   </si>
 </sst>
 </file>
@@ -472,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D305EAD-2B1E-4006-A8C6-7F0F2B69A70D}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -569,6 +575,17 @@
         <v>16</v>
       </c>
     </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>100</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add autostart evaluation feature
Added "autostart_evaluation" to settings, if true, the evaluation from "auswertung" is triggered automatically after the simulation is complete.
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9988FBC5-74D5-463C-9BC8-F8F1D27B313A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B879671-49C1-435C-A911-A81929FC27F2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>path_exe</t>
   </si>
@@ -118,6 +118,12 @@
   </si>
   <si>
     <t>CPU-Auslastung, welche unterschritten werden muss um die nächste Simulation zu starten</t>
+  </si>
+  <si>
+    <t>autostart_evaluation</t>
+  </si>
+  <si>
+    <t>1 = Die Auswertung wird automatisch nach der Simulation gestartet, 0 = Es wird lediglich simuliert, ohne die Auswertung zu starten</t>
   </si>
 </sst>
 </file>
@@ -478,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D305EAD-2B1E-4006-A8C6-7F0F2B69A70D}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -586,6 +592,17 @@
         <v>22</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Change filename of dck file in settings
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20403"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\Desktop\Tool_13062023\Basisordner\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD1748B-3617-42DF-9B59-C31B884D5C5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031F1119-0C41-4C1C-8A5D-91A29AF8FC95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>Simulationsvarianten</t>
-  </si>
-  <si>
-    <t>templateDck.dck</t>
   </si>
   <si>
     <t>C:\TRNSYS18\Exe\TrnEXE64.exe</t>
@@ -112,6 +109,9 @@
   </si>
   <si>
     <t>auto</t>
+  </si>
+  <si>
+    <t>templateDck_2.dck</t>
   </si>
 </sst>
 </file>
@@ -482,13 +482,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -496,21 +496,21 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -518,10 +518,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -533,7 +533,7 @@
         <v>1800</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -544,7 +544,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -552,21 +552,21 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change dck File template
Changed dck File to templateDck_3.dck.
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20403"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20406"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031F1119-0C41-4C1C-8A5D-91A29AF8FC95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8542FB49-30D8-42AA-BC52-6ACEE9B4F4A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -111,7 +111,7 @@
     <t>auto</t>
   </si>
   <si>
-    <t>templateDck_2.dck</t>
+    <t>templateDck_3.dck</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Move redundant files list to settings excel
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20406"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20409"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8542FB49-30D8-42AA-BC52-6ACEE9B4F4A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D515B3A0-D0BA-4099-9374-62296874B4B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>path_exe</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t>templateDck_3.dck</t>
+  </si>
+  <si>
+    <t>Liste der Dateien, die von TRNSYS produziert aber nicht benötigt werden. Diese werden aus Platzgründen nach der Simulation gelöscht. Dateinamen müssen durch ein Beistrich getrennt sein (z.B. "name1, name2, name3")</t>
+  </si>
+  <si>
+    <t>out11.txt, out8.txt, out6.txt, out7.txt, out10.txt, Speicher1_step.out</t>
+  </si>
+  <si>
+    <t>filenames_redundant</t>
   </si>
 </sst>
 </file>
@@ -472,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D305EAD-2B1E-4006-A8C6-7F0F2B69A70D}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -569,6 +578,17 @@
         <v>18</v>
       </c>
     </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Set simulation timeout using settings excel
The simulation timeout can now be set in the settings excel file and was set to 10 min.
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\TimberBioC\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45549EA4-5A7E-487F-AF33-506AC0912819}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94185BC2-5A78-4716-AC15-6684DF43B6D6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -544,8 +544,7 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <f>30*60</f>
-        <v>1800</v>
+        <v>600</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Increase simulation timeout to 1h
</commit_message>
<xml_diff>
--- a/Basisordner/Einstellungen.xlsx
+++ b/Basisordner/Einstellungen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pierre\PycharmProjects\BBSR Sommerlicher Komfort\Basisordner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682DBF24-5122-4721-A1E1-CD5D50C3DFE3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60C1B18-5F8D-4CB8-BB55-121D133CDAAF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11625" xr2:uid="{66C148C7-D7B7-490F-9EFB-309BB2932F32}"/>
   </bookViews>
@@ -538,7 +538,8 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <v>600</v>
+        <f>60*60</f>
+        <v>3600</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>

</xml_diff>